<commit_message>
GW Claim Submisssion for eform6 completed
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CA756FA-F989-4FC6-B94C-01ACFAB01501}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F70A9BF2-541A-485A-B2D7-8FE6B4BBD080}"/>
   <bookViews>
-    <workbookView xWindow="28830" yWindow="0" windowWidth="28770" windowHeight="15480" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GWCC" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3746" uniqueCount="234">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -442,15 +442,6 @@
     <t>PhysicalInjury?</t>
   </si>
   <si>
-    <t>85128943</t>
-  </si>
-  <si>
-    <t>85128944</t>
-  </si>
-  <si>
-    <t>85128946</t>
-  </si>
-  <si>
     <t>Exposure incident</t>
   </si>
   <si>
@@ -520,84 +511,9 @@
     <t>WhatareYouWearing?</t>
   </si>
   <si>
-    <t>85128949</t>
-  </si>
-  <si>
     <t>Other industry</t>
   </si>
   <si>
-    <t>85128950</t>
-  </si>
-  <si>
-    <t>85128951</t>
-  </si>
-  <si>
-    <t>85128952</t>
-  </si>
-  <si>
-    <t>85128953</t>
-  </si>
-  <si>
-    <t>85128956</t>
-  </si>
-  <si>
-    <t>85128957</t>
-  </si>
-  <si>
-    <t>85128958</t>
-  </si>
-  <si>
-    <t>85128959</t>
-  </si>
-  <si>
-    <t>85128961</t>
-  </si>
-  <si>
-    <t>85128963</t>
-  </si>
-  <si>
-    <t>85128964</t>
-  </si>
-  <si>
-    <t>85128965</t>
-  </si>
-  <si>
-    <t>85128966</t>
-  </si>
-  <si>
-    <t>85128968</t>
-  </si>
-  <si>
-    <t>85128969</t>
-  </si>
-  <si>
-    <t>85128971</t>
-  </si>
-  <si>
-    <t>85128972</t>
-  </si>
-  <si>
-    <t>85128973</t>
-  </si>
-  <si>
-    <t>85128974</t>
-  </si>
-  <si>
-    <t>85128975</t>
-  </si>
-  <si>
-    <t>85128976</t>
-  </si>
-  <si>
-    <t>85128977</t>
-  </si>
-  <si>
-    <t>85128978</t>
-  </si>
-  <si>
-    <t>85128980</t>
-  </si>
-  <si>
     <t>85128981</t>
   </si>
   <si>
@@ -605,6 +521,228 @@
   </si>
   <si>
     <t>85128983</t>
+  </si>
+  <si>
+    <t>85128984</t>
+  </si>
+  <si>
+    <t>Claim Number</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>PIN</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>32650628</t>
+  </si>
+  <si>
+    <t>01/Jan/2000</t>
+  </si>
+  <si>
+    <t>922901</t>
+  </si>
+  <si>
+    <t>85129087</t>
+  </si>
+  <si>
+    <t>32650632</t>
+  </si>
+  <si>
+    <t>569669</t>
+  </si>
+  <si>
+    <t>85129134</t>
+  </si>
+  <si>
+    <t>32650680</t>
+  </si>
+  <si>
+    <t>570172</t>
+  </si>
+  <si>
+    <t>85129135</t>
+  </si>
+  <si>
+    <t>32650682</t>
+  </si>
+  <si>
+    <t>747161</t>
+  </si>
+  <si>
+    <t>85129136</t>
+  </si>
+  <si>
+    <t>32650684</t>
+  </si>
+  <si>
+    <t>921244</t>
+  </si>
+  <si>
+    <t>85129137</t>
+  </si>
+  <si>
+    <t>32650686</t>
+  </si>
+  <si>
+    <t>072432</t>
+  </si>
+  <si>
+    <t>85129138</t>
+  </si>
+  <si>
+    <t>85129139</t>
+  </si>
+  <si>
+    <t>85129169</t>
+  </si>
+  <si>
+    <t>32650716</t>
+  </si>
+  <si>
+    <t>131505</t>
+  </si>
+  <si>
+    <t>85129170</t>
+  </si>
+  <si>
+    <t>32650718</t>
+  </si>
+  <si>
+    <t>294890</t>
+  </si>
+  <si>
+    <t>85129171</t>
+  </si>
+  <si>
+    <t>32650720</t>
+  </si>
+  <si>
+    <t>392797</t>
+  </si>
+  <si>
+    <t>85129172</t>
+  </si>
+  <si>
+    <t>32650722</t>
+  </si>
+  <si>
+    <t>578609</t>
+  </si>
+  <si>
+    <t>85129173</t>
+  </si>
+  <si>
+    <t>32650724</t>
+  </si>
+  <si>
+    <t>365781</t>
+  </si>
+  <si>
+    <t>85129174</t>
+  </si>
+  <si>
+    <t>85129175</t>
+  </si>
+  <si>
+    <t>85129176</t>
+  </si>
+  <si>
+    <t>85129177</t>
+  </si>
+  <si>
+    <t>85129178</t>
+  </si>
+  <si>
+    <t>85129179</t>
+  </si>
+  <si>
+    <t>85129180</t>
+  </si>
+  <si>
+    <t>85129181</t>
+  </si>
+  <si>
+    <t>85129182</t>
+  </si>
+  <si>
+    <t>32650726</t>
+  </si>
+  <si>
+    <t>701980</t>
+  </si>
+  <si>
+    <t>85129183</t>
+  </si>
+  <si>
+    <t>85129184</t>
+  </si>
+  <si>
+    <t>32650728</t>
+  </si>
+  <si>
+    <t>932767</t>
+  </si>
+  <si>
+    <t>85129185</t>
+  </si>
+  <si>
+    <t>32650730</t>
+  </si>
+  <si>
+    <t>050344</t>
+  </si>
+  <si>
+    <t>85129186</t>
+  </si>
+  <si>
+    <t>32650732</t>
+  </si>
+  <si>
+    <t>153486</t>
+  </si>
+  <si>
+    <t>85129187</t>
+  </si>
+  <si>
+    <t>32650734</t>
+  </si>
+  <si>
+    <t>255589</t>
+  </si>
+  <si>
+    <t>85129188</t>
+  </si>
+  <si>
+    <t>32650736</t>
+  </si>
+  <si>
+    <t>330156</t>
+  </si>
+  <si>
+    <t>85129189</t>
+  </si>
+  <si>
+    <t>85129190</t>
+  </si>
+  <si>
+    <t>32650738</t>
+  </si>
+  <si>
+    <t>894018</t>
+  </si>
+  <si>
+    <t>85129191</t>
+  </si>
+  <si>
+    <t>32650740</t>
+  </si>
+  <si>
+    <t>968191</t>
   </si>
 </sst>
 </file>
@@ -657,7 +795,47 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1064,538 +1242,588 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="16.42578125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.0"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:C1">
+    <cfRule type="duplicateValues" dxfId="16" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33828E7C-EAC4-4C86-87E0-3EB8DC303443}">
-  <dimension ref="A1:BV2"/>
+  <dimension ref="A1:BY2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="2" max="2" customWidth="true" width="16.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
     <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="13.7109375"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="14.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="48" max="48" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="49" max="51" customWidth="true" width="28.0"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="54" max="54" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="55" max="56" customWidth="true" width="33.85546875"/>
-    <col min="57" max="57" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="58" max="58" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="59" max="59" customWidth="true" width="33.85546875"/>
-    <col min="60" max="60" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="61" max="61" customWidth="true" width="25.140625"/>
-    <col min="62" max="62" customWidth="true" width="14.7109375"/>
-    <col min="63" max="63" customWidth="true" width="20.0"/>
-    <col min="64" max="64" customWidth="true" width="33.85546875"/>
-    <col min="65" max="65" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="66" max="66" customWidth="true" width="33.85546875"/>
-    <col min="67" max="68" customWidth="true" width="23.0"/>
-    <col min="69" max="69" customWidth="true" width="18.42578125"/>
-    <col min="70" max="70" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="71" max="72" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="73" max="75" customWidth="true" width="33.85546875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" width="13.7109375"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="14.42578125"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="50" max="50" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="51" max="51" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="52" max="54" customWidth="true" width="28.0"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="56" max="56" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="57" max="57" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="58" max="59" customWidth="true" width="33.85546875"/>
+    <col min="60" max="60" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="61" max="61" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="62" max="62" customWidth="true" width="33.85546875"/>
+    <col min="63" max="63" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="64" max="64" customWidth="true" width="25.140625"/>
+    <col min="65" max="65" customWidth="true" width="14.7109375"/>
+    <col min="66" max="66" customWidth="true" width="20.0"/>
+    <col min="67" max="67" customWidth="true" width="33.85546875"/>
+    <col min="68" max="68" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="69" max="69" customWidth="true" width="33.85546875"/>
+    <col min="70" max="71" customWidth="true" width="23.0"/>
+    <col min="72" max="72" customWidth="true" width="18.42578125"/>
+    <col min="73" max="73" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="74" max="75" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="76" max="78" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:74" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:77" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AX1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AY1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="BA1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="BB1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="BC1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BD1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BE1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BF1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BG1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BH1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BI1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BJ1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BK1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BL1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BM1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BN1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="BL1" s="2" t="s">
+      <c r="BO1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="BM1" s="2" t="s">
+      <c r="BP1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="BN1" s="2" t="s">
+      <c r="BQ1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="BO1" s="2" t="s">
+      <c r="BR1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="BP1" s="2" t="s">
+      <c r="BS1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BQ1" s="2" t="s">
+      <c r="BT1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="BR1" s="2" t="s">
+      <c r="BU1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="BS1" s="2" t="s">
+      <c r="BV1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="BT1" s="2" t="s">
+      <c r="BW1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="BU1" s="2" t="s">
+      <c r="BX1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="BV1" s="2" t="s">
+      <c r="BY1" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:74" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
-        <v>184</v>
+    <row r="2" spans="1:77" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>215</v>
       </c>
       <c r="B2" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="F2" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="G2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="I2" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="K2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="N2" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="M2" t="s" s="0">
+      <c r="O2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="O2" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="P2" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>28</v>
+      <c r="Q2" t="s" s="0">
+        <v>164</v>
       </c>
       <c r="R2" t="s" s="0">
         <v>80</v>
       </c>
       <c r="S2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="X2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Y2" t="s" s="0">
+      <c r="AB2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="Z2" t="s" s="0">
+      <c r="AC2" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AB2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AC2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AD2" t="s" s="0">
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AJ2" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AK2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AI2" s="1" t="s">
+      <c r="AL2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AJ2" s="1" t="s">
+      <c r="AM2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="AK2" t="s" s="0">
+      <c r="AN2" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="AL2" t="s" s="0">
+      <c r="AO2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="AM2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AN2" t="s" s="0">
+      <c r="AP2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AQ2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AO2" t="s" s="0">
+      <c r="AR2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AP2" t="s" s="0">
+      <c r="AS2" t="s" s="0">
         <v>68</v>
       </c>
-      <c r="AQ2" s="1" t="s">
+      <c r="AT2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AR2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AT2" s="1" t="s">
+      <c r="AU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AW2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AU2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AV2" t="s" s="0">
+      <c r="AX2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AW2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AX2" t="s" s="0">
+      <c r="AZ2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BA2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="AY2" t="s" s="0">
+      <c r="BB2" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="AZ2" t="s" s="0">
+      <c r="BC2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BA2" t="s" s="0">
+      <c r="BD2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BE2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BF2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BD2" t="s" s="0">
+      <c r="BG2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BE2" t="s" s="0">
+      <c r="BH2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BF2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BG2" t="s" s="0">
+      <c r="BI2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BH2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BI2" t="s" s="0">
+      <c r="BK2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BL2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BJ2" t="s" s="0">
+      <c r="BM2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BK2" t="s" s="0">
+      <c r="BN2" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BL2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BM2" t="s" s="0">
+      <c r="BO2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BP2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BN2" t="s" s="0">
+      <c r="BQ2" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="BO2" t="s" s="0">
+      <c r="BR2" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="BP2" t="s" s="0">
+      <c r="BS2" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BQ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BR2" t="s" s="0">
+      <c r="BT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="BS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BT2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BU2" t="s" s="0">
+      <c r="BV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BX2" t="s" s="0">
         <v>114</v>
       </c>
-      <c r="BV2" t="s" s="0">
+      <c r="BY2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:K1 M1:Q1 S1:XFD1">
-    <cfRule type="duplicateValues" dxfId="12" priority="3"/>
+  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
+    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1">
-    <cfRule type="duplicateValues" dxfId="11" priority="2"/>
+  <conditionalFormatting sqref="O1">
+    <cfRule type="duplicateValues" dxfId="14" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R1">
-    <cfRule type="duplicateValues" dxfId="10" priority="1"/>
+  <conditionalFormatting sqref="U1">
+    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="12" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1604,515 +1832,545 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64E6A5F-66F3-47EA-9AEB-61CD493B9923}">
-  <dimension ref="A1:BT2"/>
+  <dimension ref="A1:BW2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="33.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="33.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
     <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="35" max="35" customWidth="true" width="19.85546875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
     <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="47" max="49" customWidth="true" width="28.0"/>
-    <col min="50" max="50" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="51" max="51" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="53" max="54" customWidth="true" width="33.85546875"/>
-    <col min="55" max="55" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="56" max="56" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="57" max="57" customWidth="true" width="33.85546875"/>
-    <col min="58" max="58" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="59" max="59" customWidth="true" width="25.140625"/>
-    <col min="60" max="60" customWidth="true" width="14.7109375"/>
-    <col min="61" max="61" customWidth="true" width="20.0"/>
-    <col min="62" max="62" customWidth="true" width="33.85546875"/>
-    <col min="63" max="63" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="64" max="64" customWidth="true" width="33.85546875"/>
-    <col min="65" max="66" customWidth="true" width="23.0"/>
-    <col min="67" max="67" customWidth="true" width="18.42578125"/>
-    <col min="68" max="68" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="69" max="70" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="71" max="73" customWidth="true" width="33.85546875"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="38" max="38" customWidth="true" width="19.85546875"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="50" max="52" customWidth="true" width="28.0"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="54" max="54" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="56" max="57" customWidth="true" width="33.85546875"/>
+    <col min="58" max="58" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="59" max="59" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="60" max="60" customWidth="true" width="33.85546875"/>
+    <col min="61" max="61" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="62" max="62" customWidth="true" width="25.140625"/>
+    <col min="63" max="63" customWidth="true" width="14.7109375"/>
+    <col min="64" max="64" customWidth="true" width="20.0"/>
+    <col min="65" max="65" customWidth="true" width="33.85546875"/>
+    <col min="66" max="66" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="67" max="67" customWidth="true" width="33.85546875"/>
+    <col min="68" max="69" customWidth="true" width="23.0"/>
+    <col min="70" max="70" customWidth="true" width="18.42578125"/>
+    <col min="71" max="71" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="72" max="73" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="74" max="76" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:72" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:75" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="M1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AX1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AY1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="BA1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="BB1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="BC1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BD1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BE1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BF1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BG1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BH1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BI1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BJ1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BK1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BL1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BM1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BN1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="BL1" s="2" t="s">
+      <c r="BO1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="BM1" s="2" t="s">
+      <c r="BP1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="BN1" s="2" t="s">
+      <c r="BQ1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BO1" s="2" t="s">
+      <c r="BR1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="BP1" s="2" t="s">
+      <c r="BS1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="BQ1" s="2" t="s">
+      <c r="BT1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="BR1" s="2" t="s">
+      <c r="BU1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="BS1" s="2" t="s">
+      <c r="BV1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="BT1" s="2" t="s">
+      <c r="BW1" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:75" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>185</v>
+        <v>218</v>
       </c>
       <c r="B2" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="F2" t="s" s="0">
         <v>119</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="G2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="I2" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="K2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="N2" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="M2" t="s" s="0">
+      <c r="O2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="P2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="O2" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="P2" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>28</v>
+      <c r="Q2" t="s" s="0">
+        <v>164</v>
       </c>
       <c r="R2" t="s" s="0">
         <v>80</v>
       </c>
       <c r="S2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="X2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Y2" t="s" s="0">
+      <c r="AB2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="Z2" t="s" s="0">
+      <c r="AC2" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AB2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AC2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AD2" t="s" s="0">
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AJ2" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="AH2" t="s" s="0">
+      <c r="AK2" t="s" s="0">
         <v>123</v>
       </c>
-      <c r="AI2" t="s" s="0">
+      <c r="AL2" t="s" s="0">
         <v>124</v>
       </c>
-      <c r="AJ2" s="1" t="s">
+      <c r="AM2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AK2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AL2" t="s" s="0">
+      <c r="AN2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AO2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AM2" t="s" s="0">
+      <c r="AP2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AN2" t="s" s="0">
+      <c r="AQ2" t="s" s="0">
         <v>68</v>
       </c>
-      <c r="AO2" s="1" t="s">
+      <c r="AR2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AP2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AQ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AS2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AU2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AT2" t="s" s="0">
+      <c r="AV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AW2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AU2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AV2" t="s" s="0">
+      <c r="AX2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="AW2" t="s" s="0">
+      <c r="AZ2" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="AX2" t="s" s="0">
+      <c r="BA2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="AY2" t="s" s="0">
+      <c r="BB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="AZ2" t="s" s="0">
+      <c r="BC2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BA2" t="s" s="0">
+      <c r="BD2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BE2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BF2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BD2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BE2" t="s" s="0">
+      <c r="BG2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BH2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BF2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BG2" t="s" s="0">
+      <c r="BI2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BH2" t="s" s="0">
+      <c r="BK2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BI2" t="s" s="0">
+      <c r="BL2" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BJ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BK2" t="s" s="0">
+      <c r="BM2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BN2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BL2" t="s" s="0">
+      <c r="BO2" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="BM2" t="s" s="0">
+      <c r="BP2" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="BN2" t="s" s="0">
+      <c r="BQ2" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BO2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BP2" t="s" s="0">
+      <c r="BR2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BS2" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="BQ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BR2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BS2" t="s" s="0">
+      <c r="BT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s" s="0">
         <v>114</v>
       </c>
-      <c r="BT2" t="s" s="0">
+      <c r="BW2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:K1 M1:Q1 S1:XFD1">
-    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
+    <cfRule type="duplicateValues" dxfId="11" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1">
-    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
+  <conditionalFormatting sqref="O1">
+    <cfRule type="duplicateValues" dxfId="10" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R1">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+  <conditionalFormatting sqref="U1">
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2120,523 +2378,553 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D26FBA-7439-42B9-A201-C3C27FE83F69}">
-  <dimension ref="A1:BU2"/>
+  <dimension ref="A1:BX2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="24.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="24.28515625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.85546875"/>
     <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="34" max="35" customWidth="true" width="15.140625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="48" max="50" customWidth="true" width="28.0"/>
-    <col min="51" max="51" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="54" max="55" customWidth="true" width="33.85546875"/>
-    <col min="56" max="56" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="57" max="57" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="58" max="58" customWidth="true" width="33.85546875"/>
-    <col min="59" max="59" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="60" max="60" customWidth="true" width="25.140625"/>
-    <col min="61" max="61" customWidth="true" width="14.7109375"/>
-    <col min="62" max="62" customWidth="true" width="20.0"/>
-    <col min="63" max="63" customWidth="true" width="33.85546875"/>
-    <col min="64" max="64" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="65" max="65" customWidth="true" width="33.85546875"/>
-    <col min="66" max="67" customWidth="true" width="23.0"/>
-    <col min="68" max="68" customWidth="true" width="18.42578125"/>
-    <col min="69" max="69" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="70" max="71" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="72" max="74" customWidth="true" width="33.85546875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="37" max="38" customWidth="true" width="15.140625"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="50" max="50" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="51" max="53" customWidth="true" width="28.0"/>
+    <col min="54" max="54" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="56" max="56" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="57" max="58" customWidth="true" width="33.85546875"/>
+    <col min="59" max="59" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="60" max="60" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="61" max="61" customWidth="true" width="33.85546875"/>
+    <col min="62" max="62" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="63" max="63" customWidth="true" width="25.140625"/>
+    <col min="64" max="64" customWidth="true" width="14.7109375"/>
+    <col min="65" max="65" customWidth="true" width="20.0"/>
+    <col min="66" max="66" customWidth="true" width="33.85546875"/>
+    <col min="67" max="67" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="68" max="68" customWidth="true" width="33.85546875"/>
+    <col min="69" max="70" customWidth="true" width="23.0"/>
+    <col min="71" max="71" customWidth="true" width="18.42578125"/>
+    <col min="72" max="72" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="73" max="74" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="75" max="77" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:76" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="AX1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AV1" s="2" t="s">
+      <c r="AY1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AW1" s="2" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AX1" s="2" t="s">
+      <c r="BA1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AY1" s="2" t="s">
+      <c r="BB1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="AZ1" s="2" t="s">
+      <c r="BC1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="BA1" s="2" t="s">
+      <c r="BD1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BE1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BF1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="BD1" s="2" t="s">
+      <c r="BG1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="BE1" s="2" t="s">
+      <c r="BH1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="BF1" s="2" t="s">
+      <c r="BI1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="BG1" s="2" t="s">
+      <c r="BJ1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="BH1" s="2" t="s">
+      <c r="BK1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="BI1" s="2" t="s">
+      <c r="BL1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="BJ1" s="2" t="s">
+      <c r="BM1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="BK1" s="2" t="s">
+      <c r="BN1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="BL1" s="2" t="s">
+      <c r="BO1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="BM1" s="2" t="s">
+      <c r="BP1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="BN1" s="2" t="s">
+      <c r="BQ1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="BO1" s="2" t="s">
+      <c r="BR1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BP1" s="2" t="s">
+      <c r="BS1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="BQ1" s="2" t="s">
+      <c r="BT1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="BR1" s="2" t="s">
+      <c r="BU1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="BS1" s="2" t="s">
+      <c r="BV1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="BT1" s="2" t="s">
+      <c r="BW1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="BU1" s="2" t="s">
+      <c r="BX1" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:73" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>186</v>
+        <v>227</v>
       </c>
       <c r="B2" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="F2" t="s" s="0">
         <v>126</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="G2" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="H2" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="I2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="J2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="L2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="M2" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="L2" t="s" s="0">
+      <c r="N2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="O2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="N2" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="O2" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>28</v>
+      <c r="P2" t="s" s="0">
+        <v>164</v>
       </c>
       <c r="Q2" t="s" s="0">
         <v>80</v>
       </c>
       <c r="R2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="U2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="T2" t="s" s="0">
+      <c r="W2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="AA2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="Y2" t="s" s="0">
+      <c r="AB2" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AA2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AB2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AD2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AD2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AE2" t="s" s="0">
+      <c r="AG2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AH2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AI2" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="AG2" s="1" t="s">
+      <c r="AJ2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AK2" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="AI2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AJ2" t="s" s="0">
+      <c r="AL2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM2" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="AK2" t="s" s="0">
+      <c r="AN2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="AL2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AM2" t="s" s="0">
+      <c r="AO2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AP2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AN2" t="s" s="0">
+      <c r="AQ2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AO2" t="s" s="0">
+      <c r="AR2" t="s" s="0">
         <v>68</v>
       </c>
-      <c r="AP2" s="1" t="s">
+      <c r="AS2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AQ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AR2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AS2" s="1" t="s">
+      <c r="AT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AV2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AT2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AU2" t="s" s="0">
+      <c r="AW2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AX2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AV2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AW2" t="s" s="0">
+      <c r="AY2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AZ2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="AX2" t="s" s="0">
+      <c r="BA2" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="AY2" t="s" s="0">
+      <c r="BB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="AZ2" t="s" s="0">
+      <c r="BC2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BA2" t="s" s="0">
+      <c r="BD2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BE2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BF2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BD2" t="s" s="0">
+      <c r="BG2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BF2" t="s" s="0">
+      <c r="BH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BI2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BG2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BH2" t="s" s="0">
+      <c r="BJ2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BK2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BI2" t="s" s="0">
+      <c r="BL2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BJ2" t="s" s="0">
+      <c r="BM2" t="s" s="0">
         <v>100</v>
       </c>
-      <c r="BK2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BL2" t="s" s="0">
+      <c r="BN2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BO2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BM2" t="s" s="0">
+      <c r="BP2" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="BN2" t="s" s="0">
+      <c r="BQ2" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="BO2" t="s" s="0">
+      <c r="BR2" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BP2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BQ2" t="s" s="0">
+      <c r="BS2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BT2" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="BR2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BT2" t="s" s="0">
+      <c r="BU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s" s="0">
         <v>114</v>
       </c>
-      <c r="BU2" t="s" s="0">
+      <c r="BX2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AL1:XFD1 A1:J1 L1:P1 R1:AI1">
+  <conditionalFormatting sqref="AO1:XFD1 A1 O1:S1 U1:AL1 E1:M1">
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM1:AN1">
     <cfRule type="duplicateValues" dxfId="6" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AJ1:AK1">
+  <conditionalFormatting sqref="N1">
     <cfRule type="duplicateValues" dxfId="5" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1">
+  <conditionalFormatting sqref="T1">
     <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q1">
+  <conditionalFormatting sqref="B1:D1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2645,229 +2933,253 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{047E5626-4C4D-4FFC-85FB-69A376807120}">
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="23.28515625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
     <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="19" max="20" customWidth="true" width="18.42578125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="24" max="26" customWidth="true" width="19.5703125"/>
-    <col min="27" max="29" customWidth="true" width="17.28515625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="31" max="32" customWidth="true" width="33.85546875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="22" max="23" customWidth="true" width="18.42578125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="27" max="29" customWidth="true" width="19.5703125"/>
+    <col min="30" max="32" customWidth="true" width="17.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="34" max="35" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AB1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AG1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>187</v>
+        <v>228</v>
       </c>
       <c r="B2" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>230</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>134</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K2" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="L2" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="N2" t="s" s="0">
         <v>80</v>
       </c>
       <c r="O2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="R2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="S2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>141</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="R2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="S2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="T2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="U2" t="s" s="0">
+      <c r="W2" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="X2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="V2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="W2" t="s" s="0">
+      <c r="Y2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="X2" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="Y2" t="s" s="0">
+      <c r="AA2" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="AB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="Z2" t="s" s="0">
-        <v>148</v>
-      </c>
-      <c r="AA2" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="AB2" t="s" s="0">
-        <v>151</v>
-      </c>
       <c r="AC2" t="s" s="0">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="AD2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="AE2" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="AG2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="AH2" t="s" s="0">
         <v>114</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:XFD1">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  <conditionalFormatting sqref="A1 E1:XFD1">
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2876,223 +3188,244 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673F62D1-C22D-4ED7-B45C-1711D3211AD6}">
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="23.28515625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
     <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="19" max="20" customWidth="true" width="18.42578125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="24" max="26" customWidth="true" width="19.5703125"/>
-    <col min="27" max="29" customWidth="true" width="17.28515625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="31" max="32" customWidth="true" width="33.85546875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="22" max="23" customWidth="true" width="18.42578125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="27" max="29" customWidth="true" width="19.5703125"/>
+    <col min="30" max="32" customWidth="true" width="17.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="34" max="35" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AB1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="Q1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="AG1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="R1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="X1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A2" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>166</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="G2" t="s" s="0">
         <v>156</v>
       </c>
-      <c r="Y1" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
-        <v>179</v>
-      </c>
-      <c r="B2" t="s" s="0">
+      <c r="H2" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>160</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="I2" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="K2" t="s" s="0">
-        <v>80</v>
-      </c>
-      <c r="L2" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="N2" t="s" s="0">
         <v>80</v>
       </c>
       <c r="O2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="R2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="S2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>141</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="R2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="S2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="T2" t="s" s="0">
-        <v>144</v>
-      </c>
-      <c r="U2" t="s" s="0">
+      <c r="W2" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="X2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="V2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="W2" t="s" s="0">
+      <c r="Y2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="X2" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="Y2" t="s" s="0">
+      <c r="AA2" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="AB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="Z2" t="s" s="0">
-        <v>148</v>
-      </c>
-      <c r="AA2" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="AB2" t="s" s="0">
-        <v>151</v>
-      </c>
       <c r="AC2" t="s" s="0">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="AD2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="AE2" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>150</v>
+      </c>
+      <c r="AG2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="AH2" t="s" s="0">
         <v>114</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CAA and WT Tests
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4239" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4603" uniqueCount="253">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -770,6 +770,36 @@
   </si>
   <si>
     <t>85129343</t>
+  </si>
+  <si>
+    <t>85129344</t>
+  </si>
+  <si>
+    <t>32650893</t>
+  </si>
+  <si>
+    <t>234493</t>
+  </si>
+  <si>
+    <t>85129509</t>
+  </si>
+  <si>
+    <t>32651069</t>
+  </si>
+  <si>
+    <t>862299</t>
+  </si>
+  <si>
+    <t>85129516</t>
+  </si>
+  <si>
+    <t>85129517</t>
+  </si>
+  <si>
+    <t>32651072</t>
+  </si>
+  <si>
+    <t>895014</t>
   </si>
 </sst>
 </file>
@@ -2710,16 +2740,16 @@
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>166</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>15</v>
@@ -3099,16 +3129,16 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>166</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>133</v>
@@ -3354,16 +3384,16 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>166</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>133</v>

</xml_diff>

<commit_message>
Adding NIHL back and Appeals Tests
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{689E09CA-F413-4F20-973D-BD263674621B}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E00D7164-FA12-4DC0-8E76-843B3C7FD60B}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GWCC" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="-367" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="-3138" uniqueCount="187">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -532,12 +532,6 @@
     <t>673493</t>
   </si>
   <si>
-    <t>32651608</t>
-  </si>
-  <si>
-    <t>335647</t>
-  </si>
-  <si>
     <t>85130370</t>
   </si>
   <si>
@@ -562,9 +556,6 @@
     <t>658964</t>
   </si>
   <si>
-    <t>85130724</t>
-  </si>
-  <si>
     <t>1|May|2026</t>
   </si>
   <si>
@@ -581,6 +572,36 @@
   </si>
   <si>
     <t>479982</t>
+  </si>
+  <si>
+    <t>01/May/1992</t>
+  </si>
+  <si>
+    <t>85142521</t>
+  </si>
+  <si>
+    <t>85142522</t>
+  </si>
+  <si>
+    <t>32664481</t>
+  </si>
+  <si>
+    <t>373250</t>
+  </si>
+  <si>
+    <t>85142539</t>
+  </si>
+  <si>
+    <t>32664493</t>
+  </si>
+  <si>
+    <t>938808</t>
+  </si>
+  <si>
+    <t>85142544</t>
+  </si>
+  <si>
+    <t>85142547</t>
   </si>
 </sst>
 </file>
@@ -625,10 +646,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1080,11 +1102,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="16.42578125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.5703125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.42578125"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="7.0"/>
   </cols>
   <sheetData>
@@ -1097,6 +1119,17 @@
       </c>
       <c r="C1" s="2" t="s">
         <v>156</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="0">
+        <v>32664168</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" s="0">
+        <v>873372</v>
       </c>
     </row>
   </sheetData>
@@ -1419,16 +1452,16 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>15</v>
@@ -1578,7 +1611,7 @@
         <v>90</v>
       </c>
       <c r="BB2" t="s" s="0">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="BC2" t="s" s="0">
         <v>83</v>
@@ -1623,13 +1656,13 @@
         <v>83</v>
       </c>
       <c r="BQ2" t="s" s="0">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="BR2" t="s" s="0">
         <v>104</v>
       </c>
       <c r="BS2" t="s" s="0">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="BT2" t="s" s="0">
         <v>17</v>
@@ -1651,17 +1684,17 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
-    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="15" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1">
     <cfRule type="duplicateValues" dxfId="14" priority="3"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
+    <cfRule type="duplicateValues" dxfId="13" priority="4"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="U1">
-    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D1">
-    <cfRule type="duplicateValues" dxfId="12" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1972,7 +2005,7 @@
     </row>
     <row r="2" spans="1:75" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>159</v>
@@ -2125,7 +2158,7 @@
         <v>90</v>
       </c>
       <c r="AZ2" t="s" s="0">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="BA2" t="s" s="0">
         <v>83</v>
@@ -2170,13 +2203,13 @@
         <v>83</v>
       </c>
       <c r="BO2" t="s" s="0">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="BP2" t="s" s="0">
         <v>104</v>
       </c>
       <c r="BQ2" t="s" s="0">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="BR2" t="s" s="0">
         <v>17</v>
@@ -2198,17 +2231,17 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
-    <cfRule type="duplicateValues" dxfId="11" priority="4"/>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1">
     <cfRule type="duplicateValues" dxfId="10" priority="3"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="P1:T1 A1 V1:XFD1 E1:N1">
+    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="U1">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D1">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2521,7 +2554,7 @@
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>161</v>
@@ -2677,7 +2710,7 @@
         <v>90</v>
       </c>
       <c r="BA2" t="s" s="0">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="BB2" t="s" s="0">
         <v>83</v>
@@ -2722,13 +2755,13 @@
         <v>83</v>
       </c>
       <c r="BP2" t="s" s="0">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="BQ2" t="s" s="0">
         <v>104</v>
       </c>
       <c r="BR2" t="s" s="0">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="BS2" t="s" s="0">
         <v>17</v>
@@ -2750,20 +2783,20 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AO1:XFD1 A1 O1:S1 U1:AL1 E1:M1">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+  <conditionalFormatting sqref="B1:D1">
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1">
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T1">
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM1:AN1">
-    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T1">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:D1">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+  <conditionalFormatting sqref="AO1:XFD1 A1 O1:S1 U1:AL1 E1:M1">
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2910,16 +2943,16 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>130</v>
@@ -3165,16 +3198,16 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>130</v>

</xml_diff>

<commit_message>
OSBC Changes - partial
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -3,26 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E00D7164-FA12-4DC0-8E76-843B3C7FD60B}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A327F9B-FDAF-4F18-8144-FDA84EA90761}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GWCC" sheetId="1" r:id="rId1"/>
-    <sheet name="eForm6_PI" sheetId="2" r:id="rId2"/>
-    <sheet name="eForm6_Illness" sheetId="3" r:id="rId3"/>
-    <sheet name="eForm6_Mental" sheetId="4" r:id="rId4"/>
-    <sheet name="eForm6_Construction" sheetId="5" r:id="rId5"/>
-    <sheet name="eForm6_Other" sheetId="6" r:id="rId6"/>
+    <sheet name="eForm7_PI" sheetId="7" r:id="rId2"/>
+    <sheet name="eForm6_PI" sheetId="2" r:id="rId3"/>
+    <sheet name="eForm6_Illness" sheetId="3" r:id="rId4"/>
+    <sheet name="eForm6_Mental" sheetId="4" r:id="rId5"/>
+    <sheet name="eForm6_Construction" sheetId="5" r:id="rId6"/>
+    <sheet name="eForm6_Other" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="-3138" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294822865" uniqueCount="189">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -565,50 +566,55 @@
     <t>1|Feb|2026</t>
   </si>
   <si>
-    <t>85130734</t>
-  </si>
-  <si>
-    <t>32651978</t>
-  </si>
-  <si>
-    <t>479982</t>
-  </si>
-  <si>
     <t>01/May/1992</t>
   </si>
   <si>
-    <t>85142521</t>
-  </si>
-  <si>
-    <t>85142522</t>
-  </si>
-  <si>
-    <t>32664481</t>
-  </si>
-  <si>
-    <t>373250</t>
-  </si>
-  <si>
-    <t>85142539</t>
-  </si>
-  <si>
     <t>32664493</t>
   </si>
   <si>
     <t>938808</t>
   </si>
   <si>
-    <t>85142544</t>
-  </si>
-  <si>
     <t>85142547</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t>Report Type</t>
+  </si>
+  <si>
+    <t>Injury Category</t>
+  </si>
+  <si>
+    <t>Accident Type</t>
+  </si>
+  <si>
+    <t>Described By</t>
+  </si>
+  <si>
+    <t>Fainting</t>
+  </si>
+  <si>
+    <t>I work at the business</t>
+  </si>
+  <si>
+    <t>Mailing Address</t>
+  </si>
+  <si>
+    <t>Branch Address</t>
+  </si>
+  <si>
+    <t>Business Year</t>
+  </si>
+  <si>
+    <t>NAICS Code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -655,7 +661,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1105,9 +1121,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="16.42578125"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="12.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1122,99 +1138,187 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="0">
+      <c r="A2">
         <v>32664168</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C2" s="0">
+        <v>174</v>
+      </c>
+      <c r="C2">
         <v>873372</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:C1">
+    <cfRule type="duplicateValues" dxfId="17" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C054F313-B8A2-4709-8028-7C8E0478B7C1}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" t="s">
+        <v>185</v>
+      </c>
+      <c r="J1" t="s">
+        <v>186</v>
+      </c>
+      <c r="K1" t="s">
+        <v>187</v>
+      </c>
+      <c r="L1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>9062672</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="16" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33828E7C-EAC4-4C86-87E0-3EB8DC303443}">
   <dimension ref="A1:BY2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" customWidth="true" width="16.42578125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.5703125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="7.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="13.7109375"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="14.42578125"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="48" max="48" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="49" max="49" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="50" max="50" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="51" max="51" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="52" max="54" customWidth="true" width="28.0"/>
-    <col min="55" max="55" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="56" max="56" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="57" max="57" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="58" max="59" customWidth="true" width="33.85546875"/>
-    <col min="60" max="60" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="61" max="61" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="62" max="62" customWidth="true" width="33.85546875"/>
-    <col min="63" max="63" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="64" max="64" customWidth="true" width="25.140625"/>
-    <col min="65" max="65" customWidth="true" width="14.7109375"/>
-    <col min="66" max="66" customWidth="true" width="20.0"/>
-    <col min="67" max="67" customWidth="true" width="33.85546875"/>
-    <col min="68" max="68" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="69" max="69" customWidth="true" width="33.85546875"/>
-    <col min="70" max="71" customWidth="true" width="23.0"/>
-    <col min="72" max="72" customWidth="true" width="18.42578125"/>
-    <col min="73" max="73" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="74" max="75" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="76" max="78" customWidth="true" width="33.85546875"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="52" max="54" width="28" customWidth="1"/>
+    <col min="55" max="55" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="58" max="59" width="33.85546875" customWidth="1"/>
+    <col min="60" max="60" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="33.85546875" customWidth="1"/>
+    <col min="63" max="63" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="25.140625" customWidth="1"/>
+    <col min="65" max="65" width="14.7109375" customWidth="1"/>
+    <col min="66" max="66" width="20" customWidth="1"/>
+    <col min="67" max="67" width="33.85546875" customWidth="1"/>
+    <col min="68" max="68" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="33.85546875" customWidth="1"/>
+    <col min="70" max="71" width="23" customWidth="1"/>
+    <col min="72" max="72" width="18.42578125" customWidth="1"/>
+    <col min="73" max="73" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="74" max="75" width="19" bestFit="1" customWidth="1"/>
+    <col min="76" max="78" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:77" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1452,75 +1556,75 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>183</v>
-      </c>
-      <c r="C2" t="s" s="0">
+        <v>177</v>
+      </c>
+      <c r="B2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C2" t="s">
         <v>158</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>184</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s" s="0">
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>157</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s" s="0">
+      <c r="M2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" t="s" s="0">
+      <c r="N2" t="s">
         <v>23</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="P2" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>157</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>80</v>
       </c>
-      <c r="S2" t="s" s="0">
+      <c r="S2" t="s">
         <v>27</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="U2" t="s">
         <v>80</v>
       </c>
-      <c r="V2" t="s" s="0">
+      <c r="V2" t="s">
         <v>43</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="X2" t="s">
         <v>25</v>
       </c>
       <c r="Y2" s="1" t="s">
@@ -1532,31 +1636,31 @@
       <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>46</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AC2" t="s">
         <v>47</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AE2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s">
         <v>49</v>
       </c>
-      <c r="AH2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AI2" t="s" s="0">
+      <c r="AH2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s">
         <v>52</v>
       </c>
-      <c r="AJ2" t="s" s="0">
+      <c r="AJ2" t="s">
         <v>57</v>
       </c>
       <c r="AK2" s="1" t="s">
@@ -1568,118 +1672,118 @@
       <c r="AM2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="AN2" t="s" s="0">
+      <c r="AN2" t="s">
         <v>59</v>
       </c>
-      <c r="AO2" t="s" s="0">
+      <c r="AO2" t="s">
         <v>60</v>
       </c>
-      <c r="AP2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AQ2" t="s" s="0">
+      <c r="AP2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AQ2" t="s">
         <v>66</v>
       </c>
-      <c r="AR2" t="s" s="0">
+      <c r="AR2" t="s">
         <v>67</v>
       </c>
-      <c r="AS2" t="s" s="0">
+      <c r="AS2" t="s">
         <v>68</v>
       </c>
       <c r="AT2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AU2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AV2" t="s" s="0">
+      <c r="AU2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV2" t="s">
         <v>17</v>
       </c>
       <c r="AW2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AX2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AY2" t="s" s="0">
+      <c r="AX2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s">
         <v>76</v>
       </c>
-      <c r="AZ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BA2" t="s" s="0">
+      <c r="AZ2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BA2" t="s">
         <v>90</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BB2" t="s">
         <v>171</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BC2" t="s">
         <v>83</v>
       </c>
-      <c r="BD2" t="s" s="0">
+      <c r="BD2" t="s">
         <v>83</v>
       </c>
-      <c r="BE2" t="s" s="0">
+      <c r="BE2" t="s">
         <v>85</v>
       </c>
-      <c r="BF2" t="s" s="0">
+      <c r="BF2" t="s">
         <v>87</v>
       </c>
-      <c r="BG2" t="s" s="0">
+      <c r="BG2" t="s">
         <v>89</v>
       </c>
-      <c r="BH2" t="s" s="0">
+      <c r="BH2" t="s">
         <v>80</v>
       </c>
-      <c r="BI2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BJ2" t="s" s="0">
+      <c r="BI2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s">
         <v>83</v>
       </c>
-      <c r="BK2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BL2" t="s" s="0">
+      <c r="BK2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BL2" t="s">
         <v>83</v>
       </c>
-      <c r="BM2" t="s" s="0">
+      <c r="BM2" t="s">
         <v>98</v>
       </c>
-      <c r="BN2" t="s" s="0">
+      <c r="BN2" t="s">
         <v>99</v>
       </c>
-      <c r="BO2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BP2" t="s" s="0">
+      <c r="BO2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BP2" t="s">
         <v>83</v>
       </c>
-      <c r="BQ2" t="s" s="0">
+      <c r="BQ2" t="s">
         <v>172</v>
       </c>
-      <c r="BR2" t="s" s="0">
+      <c r="BR2" t="s">
         <v>104</v>
       </c>
-      <c r="BS2" t="s" s="0">
+      <c r="BS2" t="s">
         <v>173</v>
       </c>
-      <c r="BT2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BU2" t="s" s="0">
+      <c r="BT2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s">
         <v>107</v>
       </c>
-      <c r="BV2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BW2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BX2" t="s" s="0">
+      <c r="BV2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX2" t="s">
         <v>111</v>
       </c>
-      <c r="BY2" t="s" s="0">
+      <c r="BY2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1701,79 +1805,79 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64E6A5F-66F3-47EA-9AEB-61CD493B9923}">
   <dimension ref="A1:BW2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="33.85546875"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="38" max="38" customWidth="true" width="19.85546875"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="48" max="48" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="49" max="49" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="50" max="52" customWidth="true" width="28.0"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="54" max="54" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="55" max="55" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="56" max="57" customWidth="true" width="33.85546875"/>
-    <col min="58" max="58" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="59" max="59" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="60" max="60" customWidth="true" width="33.85546875"/>
-    <col min="61" max="61" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="62" max="62" customWidth="true" width="25.140625"/>
-    <col min="63" max="63" customWidth="true" width="14.7109375"/>
-    <col min="64" max="64" customWidth="true" width="20.0"/>
-    <col min="65" max="65" customWidth="true" width="33.85546875"/>
-    <col min="66" max="66" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="67" max="67" customWidth="true" width="33.85546875"/>
-    <col min="68" max="69" customWidth="true" width="23.0"/>
-    <col min="70" max="70" customWidth="true" width="18.42578125"/>
-    <col min="71" max="71" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="72" max="73" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="74" max="76" customWidth="true" width="33.85546875"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="19.85546875" customWidth="1"/>
+    <col min="39" max="39" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="50" max="52" width="28" customWidth="1"/>
+    <col min="53" max="53" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="57" width="33.85546875" customWidth="1"/>
+    <col min="58" max="58" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="33.85546875" customWidth="1"/>
+    <col min="61" max="61" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="25.140625" customWidth="1"/>
+    <col min="63" max="63" width="14.7109375" customWidth="1"/>
+    <col min="64" max="64" width="20" customWidth="1"/>
+    <col min="65" max="65" width="33.85546875" customWidth="1"/>
+    <col min="66" max="66" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="33.85546875" customWidth="1"/>
+    <col min="68" max="69" width="23" customWidth="1"/>
+    <col min="70" max="70" width="18.42578125" customWidth="1"/>
+    <col min="71" max="71" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="72" max="73" width="19" bestFit="1" customWidth="1"/>
+    <col min="74" max="76" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:75" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2004,76 +2108,76 @@
       </c>
     </row>
     <row r="2" spans="1:75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>163</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>159</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>158</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>160</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>116</v>
       </c>
-      <c r="G2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s" s="0">
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>157</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s" s="0">
+      <c r="M2" t="s">
         <v>22</v>
       </c>
-      <c r="N2" t="s" s="0">
+      <c r="N2" t="s">
         <v>23</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="P2" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>157</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>80</v>
       </c>
-      <c r="S2" t="s" s="0">
+      <c r="S2" t="s">
         <v>27</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="U2" t="s">
         <v>80</v>
       </c>
-      <c r="V2" t="s" s="0">
+      <c r="V2" t="s">
         <v>43</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="X2" t="s">
         <v>25</v>
       </c>
       <c r="Y2" s="1" t="s">
@@ -2085,148 +2189,148 @@
       <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>46</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AC2" t="s">
         <v>47</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AE2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s">
         <v>49</v>
       </c>
-      <c r="AH2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AI2" t="s" s="0">
+      <c r="AH2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s">
         <v>52</v>
       </c>
-      <c r="AJ2" t="s" s="0">
+      <c r="AJ2" t="s">
         <v>57</v>
       </c>
-      <c r="AK2" t="s" s="0">
+      <c r="AK2" t="s">
         <v>120</v>
       </c>
-      <c r="AL2" t="s" s="0">
+      <c r="AL2" t="s">
         <v>121</v>
       </c>
       <c r="AM2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AN2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AO2" t="s" s="0">
+      <c r="AN2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO2" t="s">
         <v>66</v>
       </c>
-      <c r="AP2" t="s" s="0">
+      <c r="AP2" t="s">
         <v>67</v>
       </c>
-      <c r="AQ2" t="s" s="0">
+      <c r="AQ2" t="s">
         <v>68</v>
       </c>
       <c r="AR2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AT2" t="s" s="0">
+      <c r="AS2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT2" t="s">
         <v>17</v>
       </c>
       <c r="AU2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AV2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AW2" t="s" s="0">
+      <c r="AV2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AW2" t="s">
         <v>76</v>
       </c>
-      <c r="AX2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AY2" t="s" s="0">
+      <c r="AX2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s">
         <v>90</v>
       </c>
-      <c r="AZ2" t="s" s="0">
+      <c r="AZ2" t="s">
         <v>171</v>
       </c>
-      <c r="BA2" t="s" s="0">
+      <c r="BA2" t="s">
         <v>83</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BB2" t="s">
         <v>83</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BC2" t="s">
         <v>85</v>
       </c>
-      <c r="BD2" t="s" s="0">
+      <c r="BD2" t="s">
         <v>87</v>
       </c>
-      <c r="BE2" t="s" s="0">
+      <c r="BE2" t="s">
         <v>89</v>
       </c>
-      <c r="BF2" t="s" s="0">
+      <c r="BF2" t="s">
         <v>80</v>
       </c>
-      <c r="BG2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BH2" t="s" s="0">
+      <c r="BG2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BH2" t="s">
         <v>83</v>
       </c>
-      <c r="BI2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BJ2" t="s" s="0">
+      <c r="BI2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s">
         <v>83</v>
       </c>
-      <c r="BK2" t="s" s="0">
+      <c r="BK2" t="s">
         <v>98</v>
       </c>
-      <c r="BL2" t="s" s="0">
+      <c r="BL2" t="s">
         <v>99</v>
       </c>
-      <c r="BM2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BN2" t="s" s="0">
+      <c r="BM2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BN2" t="s">
         <v>83</v>
       </c>
-      <c r="BO2" t="s" s="0">
+      <c r="BO2" t="s">
         <v>172</v>
       </c>
-      <c r="BP2" t="s" s="0">
+      <c r="BP2" t="s">
         <v>104</v>
       </c>
-      <c r="BQ2" t="s" s="0">
+      <c r="BQ2" t="s">
         <v>173</v>
       </c>
-      <c r="BR2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BS2" t="s" s="0">
+      <c r="BR2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BS2" t="s">
         <v>107</v>
       </c>
-      <c r="BT2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BU2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BV2" t="s" s="0">
+      <c r="BT2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s">
         <v>111</v>
       </c>
-      <c r="BW2" t="s" s="0">
+      <c r="BW2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2247,79 +2351,79 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D26FBA-7439-42B9-A201-C3C27FE83F69}">
   <dimension ref="A1:BX2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="24.28515625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="20.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.85546875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="22.85546875"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="18.5703125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="16.42578125"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="19.7109375"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="19.42578125"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="23.85546875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
-    <col min="37" max="38" customWidth="true" width="15.140625"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="13.42578125"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="16.140625"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="12.28515625"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="48" max="48" bestFit="true" customWidth="true" width="21.42578125"/>
-    <col min="49" max="49" bestFit="true" customWidth="true" width="17.28515625"/>
-    <col min="50" max="50" bestFit="true" customWidth="true" width="25.28515625"/>
-    <col min="51" max="53" customWidth="true" width="28.0"/>
-    <col min="54" max="54" bestFit="true" customWidth="true" width="23.5703125"/>
-    <col min="55" max="55" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="56" max="56" bestFit="true" customWidth="true" width="42.140625"/>
-    <col min="57" max="58" customWidth="true" width="33.85546875"/>
-    <col min="59" max="59" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="60" max="60" bestFit="true" customWidth="true" width="21.7109375"/>
-    <col min="61" max="61" customWidth="true" width="33.85546875"/>
-    <col min="62" max="62" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="63" max="63" customWidth="true" width="25.140625"/>
-    <col min="64" max="64" customWidth="true" width="14.7109375"/>
-    <col min="65" max="65" customWidth="true" width="20.0"/>
-    <col min="66" max="66" customWidth="true" width="33.85546875"/>
-    <col min="67" max="67" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="68" max="68" customWidth="true" width="33.85546875"/>
-    <col min="69" max="70" customWidth="true" width="23.0"/>
-    <col min="71" max="71" customWidth="true" width="18.42578125"/>
-    <col min="72" max="72" bestFit="true" customWidth="true" width="36.85546875"/>
-    <col min="73" max="74" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="75" max="77" customWidth="true" width="33.85546875"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="15.140625" customWidth="1"/>
+    <col min="39" max="39" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="51" max="53" width="28" customWidth="1"/>
+    <col min="54" max="54" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="42.140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="58" width="33.85546875" customWidth="1"/>
+    <col min="59" max="59" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="33.85546875" customWidth="1"/>
+    <col min="62" max="62" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="25.140625" customWidth="1"/>
+    <col min="64" max="64" width="14.7109375" customWidth="1"/>
+    <col min="65" max="65" width="20" customWidth="1"/>
+    <col min="66" max="66" width="33.85546875" customWidth="1"/>
+    <col min="67" max="67" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="33.85546875" customWidth="1"/>
+    <col min="69" max="70" width="23" customWidth="1"/>
+    <col min="71" max="71" width="18.42578125" customWidth="1"/>
+    <col min="72" max="72" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="73" max="74" width="19" bestFit="1" customWidth="1"/>
+    <col min="75" max="77" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:76" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2553,73 +2657,73 @@
       </c>
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>164</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>161</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>158</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>162</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>123</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>124</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>157</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>20</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>22</v>
       </c>
-      <c r="M2" t="s" s="0">
+      <c r="M2" t="s">
         <v>23</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="O2" t="s" s="0">
+      <c r="O2" t="s">
         <v>26</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="P2" t="s">
         <v>157</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>80</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>27</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="T2" t="s" s="0">
+      <c r="T2" t="s">
         <v>80</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="U2" t="s">
         <v>43</v>
       </c>
       <c r="V2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="W2" t="s" s="0">
+      <c r="W2" t="s">
         <v>25</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -2631,31 +2735,31 @@
       <c r="Z2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AA2" t="s" s="0">
+      <c r="AA2" t="s">
         <v>46</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>47</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AD2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AE2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AD2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s">
         <v>49</v>
       </c>
-      <c r="AG2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AH2" t="s" s="0">
+      <c r="AG2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH2" t="s">
         <v>52</v>
       </c>
-      <c r="AI2" t="s" s="0">
+      <c r="AI2" t="s">
         <v>57</v>
       </c>
       <c r="AJ2" s="1" t="s">
@@ -2667,118 +2771,118 @@
       <c r="AL2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AM2" t="s" s="0">
+      <c r="AM2" t="s">
         <v>59</v>
       </c>
-      <c r="AN2" t="s" s="0">
+      <c r="AN2" t="s">
         <v>60</v>
       </c>
-      <c r="AO2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AP2" t="s" s="0">
+      <c r="AO2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AP2" t="s">
         <v>66</v>
       </c>
-      <c r="AQ2" t="s" s="0">
+      <c r="AQ2" t="s">
         <v>67</v>
       </c>
-      <c r="AR2" t="s" s="0">
+      <c r="AR2" t="s">
         <v>68</v>
       </c>
       <c r="AS2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AT2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AU2" t="s" s="0">
+      <c r="AT2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AU2" t="s">
         <v>17</v>
       </c>
       <c r="AV2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AW2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AX2" t="s" s="0">
+      <c r="AW2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AX2" t="s">
         <v>76</v>
       </c>
-      <c r="AY2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="AZ2" t="s" s="0">
+      <c r="AY2" t="s">
+        <v>17</v>
+      </c>
+      <c r="AZ2" t="s">
         <v>90</v>
       </c>
-      <c r="BA2" t="s" s="0">
+      <c r="BA2" t="s">
         <v>171</v>
       </c>
-      <c r="BB2" t="s" s="0">
+      <c r="BB2" t="s">
         <v>83</v>
       </c>
-      <c r="BC2" t="s" s="0">
+      <c r="BC2" t="s">
         <v>83</v>
       </c>
-      <c r="BD2" t="s" s="0">
+      <c r="BD2" t="s">
         <v>85</v>
       </c>
-      <c r="BE2" t="s" s="0">
+      <c r="BE2" t="s">
         <v>87</v>
       </c>
-      <c r="BF2" t="s" s="0">
+      <c r="BF2" t="s">
         <v>89</v>
       </c>
-      <c r="BG2" t="s" s="0">
+      <c r="BG2" t="s">
         <v>80</v>
       </c>
-      <c r="BH2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BI2" t="s" s="0">
+      <c r="BH2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BI2" t="s">
         <v>83</v>
       </c>
-      <c r="BJ2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BK2" t="s" s="0">
+      <c r="BJ2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BK2" t="s">
         <v>83</v>
       </c>
-      <c r="BL2" t="s" s="0">
+      <c r="BL2" t="s">
         <v>98</v>
       </c>
-      <c r="BM2" t="s" s="0">
+      <c r="BM2" t="s">
         <v>99</v>
       </c>
-      <c r="BN2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BO2" t="s" s="0">
+      <c r="BN2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BO2" t="s">
         <v>83</v>
       </c>
-      <c r="BP2" t="s" s="0">
+      <c r="BP2" t="s">
         <v>172</v>
       </c>
-      <c r="BQ2" t="s" s="0">
+      <c r="BQ2" t="s">
         <v>104</v>
       </c>
-      <c r="BR2" t="s" s="0">
+      <c r="BR2" t="s">
         <v>173</v>
       </c>
-      <c r="BS2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BT2" t="s" s="0">
+      <c r="BS2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BT2" t="s">
         <v>107</v>
       </c>
-      <c r="BU2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BV2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="BW2" t="s" s="0">
+      <c r="BU2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s">
         <v>111</v>
       </c>
-      <c r="BX2" t="s" s="0">
+      <c r="BX2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2802,39 +2906,39 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{047E5626-4C4D-4FFC-85FB-69A376807120}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="22" max="23" customWidth="true" width="18.42578125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="27" max="29" customWidth="true" width="19.5703125"/>
-    <col min="30" max="32" customWidth="true" width="17.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="34" max="35" customWidth="true" width="33.85546875"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="18.42578125" customWidth="1"/>
+    <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="29" width="19.5703125" customWidth="1"/>
+    <col min="30" max="32" width="17.28515625" customWidth="1"/>
+    <col min="33" max="33" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2942,58 +3046,58 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>165</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>166</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>158</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>167</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>130</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>138</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>131</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>20</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="N2" t="s" s="0">
+      <c r="N2" t="s">
         <v>80</v>
       </c>
-      <c r="O2" t="s" s="0">
+      <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>80</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>43</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -3002,46 +3106,46 @@
       <c r="T2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="U2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="V2" t="s" s="0">
+      <c r="U2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s">
         <v>138</v>
       </c>
-      <c r="W2" t="s" s="0">
+      <c r="W2" t="s">
         <v>138</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="X2" t="s">
         <v>49</v>
       </c>
-      <c r="Y2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="Z2" t="s" s="0">
+      <c r="Y2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s">
         <v>52</v>
       </c>
-      <c r="AA2" t="s" s="0">
+      <c r="AA2" t="s">
         <v>140</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>83</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AC2" t="s">
         <v>142</v>
       </c>
-      <c r="AD2" t="s" s="0">
+      <c r="AD2" t="s">
         <v>43</v>
       </c>
-      <c r="AE2" t="s" s="0">
+      <c r="AE2" t="s">
         <v>145</v>
       </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AF2" t="s">
         <v>147</v>
       </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AG2" t="s">
         <v>43</v>
       </c>
-      <c r="AH2" t="s" s="0">
+      <c r="AH2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -3057,39 +3161,39 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673F62D1-C22D-4ED7-B45C-1711D3211AD6}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="22" max="23" customWidth="true" width="18.42578125"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
-    <col min="27" max="29" customWidth="true" width="19.5703125"/>
-    <col min="30" max="32" customWidth="true" width="17.28515625"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
-    <col min="34" max="35" customWidth="true" width="33.85546875"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="18.42578125" customWidth="1"/>
+    <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="29" width="19.5703125" customWidth="1"/>
+    <col min="30" max="32" width="17.28515625" customWidth="1"/>
+    <col min="33" max="33" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3197,58 +3301,58 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>168</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>169</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>158</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>170</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>130</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>138</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>153</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>20</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="N2" t="s" s="0">
+      <c r="N2" t="s">
         <v>80</v>
       </c>
-      <c r="O2" t="s" s="0">
+      <c r="O2" t="s">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>80</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>43</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -3257,46 +3361,46 @@
       <c r="T2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="U2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="V2" t="s" s="0">
+      <c r="U2" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s">
         <v>138</v>
       </c>
-      <c r="W2" t="s" s="0">
+      <c r="W2" t="s">
         <v>138</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="X2" t="s">
         <v>49</v>
       </c>
-      <c r="Y2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="Z2" t="s" s="0">
+      <c r="Y2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s">
         <v>52</v>
       </c>
-      <c r="AA2" t="s" s="0">
+      <c r="AA2" t="s">
         <v>140</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>83</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AC2" t="s">
         <v>142</v>
       </c>
-      <c r="AD2" t="s" s="0">
+      <c r="AD2" t="s">
         <v>43</v>
       </c>
-      <c r="AE2" t="s" s="0">
+      <c r="AE2" t="s">
         <v>145</v>
       </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AF2" t="s">
         <v>147</v>
       </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AG2" t="s">
         <v>43</v>
       </c>
-      <c r="AH2" t="s" s="0">
+      <c r="AH2" t="s">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
OSBC Changes E2E with some xml file update
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A327F9B-FDAF-4F18-8144-FDA84EA90761}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80A7960F-AB54-4A98-BF81-28F5BF5AFFC6}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294822865" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="244">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -575,9 +575,6 @@
     <t>938808</t>
   </si>
   <si>
-    <t>85142547</t>
-  </si>
-  <si>
     <t>Account Number</t>
   </si>
   <si>
@@ -609,12 +606,183 @@
   </si>
   <si>
     <t>NAICS Code</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>Language of Service</t>
+  </si>
+  <si>
+    <t>SIN</t>
+  </si>
+  <si>
+    <t>140 Erskine Avenue|Toronto|Ontario|M4P 1Z2</t>
+  </si>
+  <si>
+    <t>Job Title</t>
+  </si>
+  <si>
+    <t>Emp Start Date</t>
+  </si>
+  <si>
+    <t>Emp Years</t>
+  </si>
+  <si>
+    <t>Emp Months</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t># Employees</t>
+  </si>
+  <si>
+    <t>Union?</t>
+  </si>
+  <si>
+    <t>IsSpouseRelavtive</t>
+  </si>
+  <si>
+    <t>EmployerRelation</t>
+  </si>
+  <si>
+    <t>Supervisor Contact</t>
+  </si>
+  <si>
+    <t>S First|S Last|6478787777|English</t>
+  </si>
+  <si>
+    <t>WhatHappenedInput</t>
+  </si>
+  <si>
+    <t>Injury Date</t>
+  </si>
+  <si>
+    <t>Body Parts</t>
+  </si>
+  <si>
+    <t>Ear(s)</t>
+  </si>
+  <si>
+    <t>EmployerKnownDate</t>
+  </si>
+  <si>
+    <t>reported to?</t>
+  </si>
+  <si>
+    <t>Kiran|Kangula|6478777777|English</t>
+  </si>
+  <si>
+    <t>Witness</t>
+  </si>
+  <si>
+    <t>Prior Conditions</t>
+  </si>
+  <si>
+    <t>Third Party</t>
+  </si>
+  <si>
+    <t>Objection</t>
+  </si>
+  <si>
+    <t>HealthCare</t>
+  </si>
+  <si>
+    <t>LOE</t>
+  </si>
+  <si>
+    <t>Type of Work</t>
+  </si>
+  <si>
+    <t>Regular</t>
+  </si>
+  <si>
+    <t>Wage Loss</t>
+  </si>
+  <si>
+    <t>1102322</t>
+  </si>
+  <si>
+    <t>8045 SOUTH BAY RD, SUDBURY, ON, P3E 1A1, CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same as mailing address </t>
+  </si>
+  <si>
+    <t>623110</t>
+  </si>
+  <si>
+    <t>6478444444</t>
+  </si>
+  <si>
+    <t>1/Jan/1990</t>
+  </si>
+  <si>
+    <t>1/Jan/2020</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Yes|Clinic|1/Mar/2025|1/Mar/2025</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>1/Feb/2024</t>
+  </si>
+  <si>
+    <t>1/Mar/2024</t>
+  </si>
+  <si>
+    <t>85142631</t>
+  </si>
+  <si>
+    <t>85142652</t>
+  </si>
+  <si>
+    <t>Autodcmqi</t>
+  </si>
+  <si>
+    <t>Testbtezw</t>
+  </si>
+  <si>
+    <t>85142653</t>
+  </si>
+  <si>
+    <t>85142655</t>
+  </si>
+  <si>
+    <t>Autowfsdb</t>
+  </si>
+  <si>
+    <t>Testhlwmg</t>
+  </si>
+  <si>
+    <t>32664620</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/mmm/yyyy"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -652,11 +820,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1121,9 +1290,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="16.42578125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="12.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1138,13 +1307,13 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>32664168</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <v>873372</v>
       </c>
     </row>
@@ -1158,86 +1327,314 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C054F313-B8A2-4709-8028-7C8E0478B7C1}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.28515625" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="3" max="3" customWidth="true" width="17.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="12.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="15.28515625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="13.140625"/>
+    <col min="13" max="13" customWidth="true" width="15.28515625"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="10.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="14.5703125"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="12.140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="18.7109375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="43.28515625"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="10.0"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="12.0"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="31.140625"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="10.7109375"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="20.0"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="32.5703125"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" width="15.42578125"/>
+    <col min="41" max="41" customWidth="true" width="12.0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s" s="0">
         <v>180</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>184</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>187</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="R1" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="S1" t="s" s="0">
+        <v>192</v>
+      </c>
+      <c r="T1" t="s" s="0">
+        <v>193</v>
+      </c>
+      <c r="U1" t="s" s="0">
+        <v>194</v>
+      </c>
+      <c r="V1" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="W1" t="s" s="0">
+        <v>196</v>
+      </c>
+      <c r="X1" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="Y1" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="Z1" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="AA1" t="s" s="0">
+        <v>205</v>
+      </c>
+      <c r="AB1" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="AC1" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="AD1" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="AE1" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="AF1" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="AG1" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="AH1" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="AI1" t="s" s="0">
+        <v>211</v>
+      </c>
+      <c r="AJ1" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="AK1" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="AL1" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="AM1" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="AN1" t="s" s="0">
+        <v>217</v>
+      </c>
+      <c r="AO1" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="AP1" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="AQ1" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="AR1" t="s" s="0">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+      <c r="A2" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>240</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>243</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="F1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="F2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>182</v>
       </c>
-      <c r="H1" t="s">
-        <v>84</v>
-      </c>
-      <c r="I1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J1" t="s">
-        <v>186</v>
-      </c>
-      <c r="K1" t="s">
-        <v>187</v>
-      </c>
-      <c r="L1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>9062672</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s" s="0">
         <v>183</v>
       </c>
-      <c r="H2" t="s">
-        <v>184</v>
+      <c r="J2" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>238</v>
+      </c>
+      <c r="P2" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="R2" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="T2" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="V2" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="W2" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="Z2" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="AA2" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="AB2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AC2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AD2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AE2" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="AG2" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="AH2" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="AJ2" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="AK2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AL2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AM2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AN2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AO2" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="AP2" t="s" s="0">
+        <v>138</v>
+      </c>
+      <c r="AQ2" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="AR2" t="s" s="0">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:B1">
+  <conditionalFormatting sqref="A1:C1">
     <cfRule type="duplicateValues" dxfId="16" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1249,76 +1646,76 @@
   <dimension ref="A1:BY2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="9" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="52" max="54" width="28" customWidth="1"/>
-    <col min="55" max="55" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="58" max="59" width="33.85546875" customWidth="1"/>
-    <col min="60" max="60" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="33.85546875" customWidth="1"/>
-    <col min="63" max="63" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="25.140625" customWidth="1"/>
-    <col min="65" max="65" width="14.7109375" customWidth="1"/>
-    <col min="66" max="66" width="20" customWidth="1"/>
-    <col min="67" max="67" width="33.85546875" customWidth="1"/>
-    <col min="68" max="68" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="33.85546875" customWidth="1"/>
-    <col min="70" max="71" width="23" customWidth="1"/>
-    <col min="72" max="72" width="18.42578125" customWidth="1"/>
-    <col min="73" max="73" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="74" max="75" width="19" bestFit="1" customWidth="1"/>
-    <col min="76" max="78" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="2" max="2" customWidth="true" width="16.42578125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="11.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="8" max="8" customWidth="true" width="15.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" width="13.7109375"/>
+    <col min="38" max="38" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="14.42578125"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="50" max="50" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="51" max="51" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="52" max="54" customWidth="true" width="28.0"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="56" max="56" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="57" max="57" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="58" max="59" customWidth="true" width="33.85546875"/>
+    <col min="60" max="60" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="61" max="61" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="62" max="62" customWidth="true" width="33.85546875"/>
+    <col min="63" max="63" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="64" max="64" customWidth="true" width="25.140625"/>
+    <col min="65" max="65" customWidth="true" width="14.7109375"/>
+    <col min="66" max="66" customWidth="true" width="20.0"/>
+    <col min="67" max="67" customWidth="true" width="33.85546875"/>
+    <col min="68" max="68" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="69" max="69" customWidth="true" width="33.85546875"/>
+    <col min="70" max="71" customWidth="true" width="23.0"/>
+    <col min="72" max="72" customWidth="true" width="18.42578125"/>
+    <col min="73" max="73" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="74" max="75" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="76" max="78" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:77" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1556,75 +1953,75 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B2" t="s" s="0">
         <v>175</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>176</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="G2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>23</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" t="s" s="0">
         <v>27</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" t="s" s="0">
         <v>25</v>
       </c>
       <c r="Y2" s="1" t="s">
@@ -1636,31 +2033,31 @@
       <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" t="s" s="0">
         <v>47</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AE2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AG2" t="s">
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AH2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI2" t="s">
+      <c r="AH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AJ2" t="s" s="0">
         <v>57</v>
       </c>
       <c r="AK2" s="1" t="s">
@@ -1672,118 +2069,118 @@
       <c r="AM2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AN2" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AO2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="AP2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AQ2" t="s">
+      <c r="AP2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AQ2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AR2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AS2" t="s" s="0">
         <v>68</v>
       </c>
       <c r="AT2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AU2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AV2" t="s">
+      <c r="AU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AV2" t="s" s="0">
         <v>17</v>
       </c>
       <c r="AW2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AX2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AY2" t="s">
+      <c r="AX2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AZ2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BA2" t="s">
+      <c r="AZ2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BA2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BB2" t="s" s="0">
         <v>171</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BC2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BD2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BE2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BF2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BG2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BH2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BI2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BJ2" t="s">
+      <c r="BI2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BK2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BL2" t="s">
+      <c r="BK2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BL2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BM2" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BN2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BO2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BP2" t="s">
+      <c r="BO2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BP2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BQ2" t="s" s="0">
         <v>172</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BR2" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="BS2" t="s" s="0">
         <v>173</v>
       </c>
-      <c r="BT2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BU2" t="s">
+      <c r="BT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="BV2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BX2" t="s">
+      <c r="BV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BX2" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="BY2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
@@ -1810,74 +2207,74 @@
   <dimension ref="A1:BW2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="19.85546875" customWidth="1"/>
-    <col min="39" max="39" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="50" max="52" width="28" customWidth="1"/>
-    <col min="53" max="53" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="33.85546875" customWidth="1"/>
-    <col min="58" max="58" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="33.85546875" customWidth="1"/>
-    <col min="61" max="61" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="25.140625" customWidth="1"/>
-    <col min="63" max="63" width="14.7109375" customWidth="1"/>
-    <col min="64" max="64" width="20" customWidth="1"/>
-    <col min="65" max="65" width="33.85546875" customWidth="1"/>
-    <col min="66" max="66" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="33.85546875" customWidth="1"/>
-    <col min="68" max="69" width="23" customWidth="1"/>
-    <col min="70" max="70" width="18.42578125" customWidth="1"/>
-    <col min="71" max="71" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="72" max="73" width="19" bestFit="1" customWidth="1"/>
-    <col min="74" max="76" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="33.85546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="37" max="37" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="38" max="38" customWidth="true" width="19.85546875"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="50" max="52" customWidth="true" width="28.0"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="54" max="54" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="56" max="57" customWidth="true" width="33.85546875"/>
+    <col min="58" max="58" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="59" max="59" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="60" max="60" customWidth="true" width="33.85546875"/>
+    <col min="61" max="61" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="62" max="62" customWidth="true" width="25.140625"/>
+    <col min="63" max="63" customWidth="true" width="14.7109375"/>
+    <col min="64" max="64" customWidth="true" width="20.0"/>
+    <col min="65" max="65" customWidth="true" width="33.85546875"/>
+    <col min="66" max="66" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="67" max="67" customWidth="true" width="33.85546875"/>
+    <col min="68" max="69" customWidth="true" width="23.0"/>
+    <col min="70" max="70" customWidth="true" width="18.42578125"/>
+    <col min="71" max="71" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="72" max="73" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="74" max="76" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:75" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2108,76 +2505,76 @@
       </c>
     </row>
     <row r="2" spans="1:75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>159</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>160</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="G2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>23</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" t="s" s="0">
         <v>27</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" t="s" s="0">
         <v>25</v>
       </c>
       <c r="Y2" s="1" t="s">
@@ -2189,148 +2586,148 @@
       <c r="AA2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" t="s" s="0">
         <v>47</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AE2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AG2" t="s">
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AG2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AH2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AI2" t="s">
+      <c r="AH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AI2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AJ2" t="s" s="0">
         <v>57</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AK2" t="s" s="0">
         <v>120</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AL2" t="s" s="0">
         <v>121</v>
       </c>
       <c r="AM2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AN2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AO2" t="s">
+      <c r="AN2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AO2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AP2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AQ2" t="s" s="0">
         <v>68</v>
       </c>
       <c r="AR2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AS2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AT2" t="s">
+      <c r="AS2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AT2" t="s" s="0">
         <v>17</v>
       </c>
       <c r="AU2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AV2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AW2" t="s">
+      <c r="AV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AW2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AX2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AY2" t="s">
+      <c r="AX2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AY2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="AZ2" t="s" s="0">
         <v>171</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BA2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BC2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BD2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BE2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BF2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BG2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BH2" t="s">
+      <c r="BG2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BH2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BI2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BJ2" t="s">
+      <c r="BI2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BJ2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BK2" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BL2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BM2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BN2" t="s">
+      <c r="BM2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BN2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BO2" t="s" s="0">
         <v>172</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BP2" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BQ2" t="s" s="0">
         <v>173</v>
       </c>
-      <c r="BR2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BS2" t="s">
+      <c r="BR2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BS2" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="BT2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BV2" t="s">
+      <c r="BT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="BW2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
@@ -2356,74 +2753,74 @@
   <dimension ref="A1:BX2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="15.140625" customWidth="1"/>
-    <col min="39" max="39" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="9" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="51" max="53" width="28" customWidth="1"/>
-    <col min="54" max="54" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="58" width="33.85546875" customWidth="1"/>
-    <col min="59" max="59" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="33.85546875" customWidth="1"/>
-    <col min="62" max="62" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="25.140625" customWidth="1"/>
-    <col min="64" max="64" width="14.7109375" customWidth="1"/>
-    <col min="65" max="65" width="20" customWidth="1"/>
-    <col min="66" max="66" width="33.85546875" customWidth="1"/>
-    <col min="67" max="67" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="33.85546875" customWidth="1"/>
-    <col min="69" max="70" width="23" customWidth="1"/>
-    <col min="71" max="71" width="18.42578125" customWidth="1"/>
-    <col min="72" max="72" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="73" max="74" width="19" bestFit="1" customWidth="1"/>
-    <col min="75" max="77" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="24.28515625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="20.42578125"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" width="18.5703125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="16.42578125"/>
+    <col min="25" max="25" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.7109375"/>
+    <col min="27" max="27" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="28" max="28" bestFit="true" customWidth="true" width="19.42578125"/>
+    <col min="29" max="29" bestFit="true" customWidth="true" width="23.85546875"/>
+    <col min="30" max="30" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="32" max="32" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="34" max="34" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="35" max="35" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="36" max="36" bestFit="true" customWidth="true" width="15.140625"/>
+    <col min="37" max="38" customWidth="true" width="15.140625"/>
+    <col min="39" max="39" bestFit="true" customWidth="true" width="13.42578125"/>
+    <col min="40" max="40" bestFit="true" customWidth="true" width="9.0"/>
+    <col min="41" max="41" bestFit="true" customWidth="true" width="16.140625"/>
+    <col min="42" max="42" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="43" max="43" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="44" max="44" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="45" max="45" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="46" max="46" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="47" max="47" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="48" max="48" bestFit="true" customWidth="true" width="21.42578125"/>
+    <col min="49" max="49" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="50" max="50" bestFit="true" customWidth="true" width="25.28515625"/>
+    <col min="51" max="53" customWidth="true" width="28.0"/>
+    <col min="54" max="54" bestFit="true" customWidth="true" width="23.5703125"/>
+    <col min="55" max="55" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="56" max="56" bestFit="true" customWidth="true" width="42.140625"/>
+    <col min="57" max="58" customWidth="true" width="33.85546875"/>
+    <col min="59" max="59" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="60" max="60" bestFit="true" customWidth="true" width="21.7109375"/>
+    <col min="61" max="61" customWidth="true" width="33.85546875"/>
+    <col min="62" max="62" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="63" max="63" customWidth="true" width="25.140625"/>
+    <col min="64" max="64" customWidth="true" width="14.7109375"/>
+    <col min="65" max="65" customWidth="true" width="20.0"/>
+    <col min="66" max="66" customWidth="true" width="33.85546875"/>
+    <col min="67" max="67" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="68" max="68" customWidth="true" width="33.85546875"/>
+    <col min="69" max="70" customWidth="true" width="23.0"/>
+    <col min="71" max="71" customWidth="true" width="18.42578125"/>
+    <col min="72" max="72" bestFit="true" customWidth="true" width="36.85546875"/>
+    <col min="73" max="74" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="75" max="77" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:76" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2657,73 +3054,73 @@
       </c>
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>161</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>123</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>124</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" t="s" s="0">
         <v>23</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" t="s" s="0">
         <v>157</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" t="s" s="0">
         <v>27</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="V2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" t="s" s="0">
         <v>25</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -2735,31 +3132,31 @@
       <c r="Z2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" t="s" s="0">
         <v>47</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AD2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AD2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AE2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AF2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="AG2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AH2" t="s">
+      <c r="AG2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AH2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AI2" t="s" s="0">
         <v>57</v>
       </c>
       <c r="AJ2" s="1" t="s">
@@ -2771,118 +3168,118 @@
       <c r="AL2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AM2" t="s" s="0">
         <v>59</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AN2" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="AO2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AP2" t="s">
+      <c r="AO2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AP2" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AQ2" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AR2" t="s" s="0">
         <v>68</v>
       </c>
       <c r="AS2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AT2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AU2" t="s">
+      <c r="AT2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AU2" t="s" s="0">
         <v>17</v>
       </c>
       <c r="AV2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AW2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AX2" t="s">
+      <c r="AW2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AX2" t="s" s="0">
         <v>76</v>
       </c>
-      <c r="AY2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AZ2" t="s">
+      <c r="AY2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="AZ2" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BA2" t="s" s="0">
         <v>171</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BC2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BD2" t="s" s="0">
         <v>85</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BE2" t="s" s="0">
         <v>87</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BF2" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BG2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="BH2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BI2" t="s">
+      <c r="BH2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BI2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BJ2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BK2" t="s">
+      <c r="BJ2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BK2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BL2" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BM2" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="BN2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BO2" t="s">
+      <c r="BN2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BO2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BP2" t="s" s="0">
         <v>172</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BQ2" t="s" s="0">
         <v>104</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BR2" t="s" s="0">
         <v>173</v>
       </c>
-      <c r="BS2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BT2" t="s">
+      <c r="BS2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BT2" t="s" s="0">
         <v>107</v>
       </c>
-      <c r="BU2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>17</v>
-      </c>
-      <c r="BW2" t="s">
+      <c r="BU2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BV2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="BW2" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="BX2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
@@ -2911,34 +3308,34 @@
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="18.42578125" customWidth="1"/>
-    <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="29" width="19.5703125" customWidth="1"/>
-    <col min="30" max="32" width="17.28515625" customWidth="1"/>
-    <col min="33" max="33" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="22" max="23" customWidth="true" width="18.42578125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="27" max="29" customWidth="true" width="19.5703125"/>
+    <col min="30" max="32" customWidth="true" width="17.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="34" max="35" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3046,58 +3443,58 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>165</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>166</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>167</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>130</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>23</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" t="s" s="0">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -3106,46 +3503,46 @@
       <c r="T2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="U2" t="s">
-        <v>17</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="U2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="Y2" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="Y2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" t="s" s="0">
         <v>140</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" t="s" s="0">
         <v>142</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AD2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AE2" t="s" s="0">
         <v>145</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AF2" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AG2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AH2" t="s" s="0">
         <v>111</v>
       </c>
     </row>
@@ -3166,34 +3563,34 @@
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="18.42578125" customWidth="1"/>
-    <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="29" width="19.5703125" customWidth="1"/>
-    <col min="30" max="32" width="17.28515625" customWidth="1"/>
-    <col min="33" max="33" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="17.7109375"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="13.85546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="4.140625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="17.0"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="23.28515625"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="10.140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="14.140625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.42578125"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="7.5703125"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="14.7109375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="14.85546875"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="22.85546875"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="47.42578125"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="8.0"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="15.7109375"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="22" max="23" customWidth="true" width="18.42578125"/>
+    <col min="24" max="24" bestFit="true" customWidth="true" width="17.42578125"/>
+    <col min="26" max="26" bestFit="true" customWidth="true" width="19.5703125"/>
+    <col min="27" max="29" customWidth="true" width="19.5703125"/>
+    <col min="30" max="32" customWidth="true" width="17.28515625"/>
+    <col min="33" max="33" bestFit="true" customWidth="true" width="19.85546875"/>
+    <col min="34" max="35" customWidth="true" width="33.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3301,58 +3698,58 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>168</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>169</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>170</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>130</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" t="s" s="0">
         <v>23</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" t="s" s="0">
         <v>27</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" t="s" s="0">
         <v>80</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" t="s" s="0">
         <v>43</v>
       </c>
       <c r="S2" s="1" t="s">
@@ -3361,46 +3758,46 @@
       <c r="T2" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="U2" t="s">
-        <v>17</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="U2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" t="s" s="0">
         <v>138</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="Y2" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="Y2" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="Z2" t="s" s="0">
         <v>52</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" t="s" s="0">
         <v>140</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" t="s" s="0">
         <v>142</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AD2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AE2" t="s" s="0">
         <v>145</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AF2" t="s" s="0">
         <v>147</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AG2" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AH2" t="s" s="0">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
with Retry 3 times when test fails
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="264">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -774,6 +774,66 @@
   </si>
   <si>
     <t>32664620</t>
+  </si>
+  <si>
+    <t>85142660</t>
+  </si>
+  <si>
+    <t>32664631</t>
+  </si>
+  <si>
+    <t>575821</t>
+  </si>
+  <si>
+    <t>85142662</t>
+  </si>
+  <si>
+    <t>32664635</t>
+  </si>
+  <si>
+    <t>060368</t>
+  </si>
+  <si>
+    <t>85142664</t>
+  </si>
+  <si>
+    <t>32664638</t>
+  </si>
+  <si>
+    <t>237627</t>
+  </si>
+  <si>
+    <t>85142665</t>
+  </si>
+  <si>
+    <t>85142667</t>
+  </si>
+  <si>
+    <t>32664643</t>
+  </si>
+  <si>
+    <t>590865</t>
+  </si>
+  <si>
+    <t>85142668</t>
+  </si>
+  <si>
+    <t>85142669</t>
+  </si>
+  <si>
+    <t>Autolsvqq</t>
+  </si>
+  <si>
+    <t>Testveaou</t>
+  </si>
+  <si>
+    <t>85142670</t>
+  </si>
+  <si>
+    <t>32664651</t>
+  </si>
+  <si>
+    <t>301850</t>
   </si>
 </sst>
 </file>
@@ -1504,7 +1564,7 @@
         <v>223</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>243</v>
@@ -1953,16 +2013,16 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>239</v>
+        <v>261</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>175</v>
+        <v>262</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>176</v>
+        <v>263</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>15</v>

</xml_diff>

<commit_message>
Results File Management with Environments
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3206" uniqueCount="307">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -834,6 +834,135 @@
   </si>
   <si>
     <t>301850</t>
+  </si>
+  <si>
+    <t>85142671</t>
+  </si>
+  <si>
+    <t>Autoybkzz</t>
+  </si>
+  <si>
+    <t>Testpnlry</t>
+  </si>
+  <si>
+    <t>85142697</t>
+  </si>
+  <si>
+    <t>85142698</t>
+  </si>
+  <si>
+    <t>85142699</t>
+  </si>
+  <si>
+    <t>85142700</t>
+  </si>
+  <si>
+    <t>Autosxtdx</t>
+  </si>
+  <si>
+    <t>Testjjtni</t>
+  </si>
+  <si>
+    <t>85142703</t>
+  </si>
+  <si>
+    <t>32664708</t>
+  </si>
+  <si>
+    <t>993630</t>
+  </si>
+  <si>
+    <t>85142716</t>
+  </si>
+  <si>
+    <t>Autoglyvm</t>
+  </si>
+  <si>
+    <t>Testkskic</t>
+  </si>
+  <si>
+    <t>85142727</t>
+  </si>
+  <si>
+    <t>Autopafdk</t>
+  </si>
+  <si>
+    <t>Testpmrkf</t>
+  </si>
+  <si>
+    <t>85142730</t>
+  </si>
+  <si>
+    <t>Autoxabxq</t>
+  </si>
+  <si>
+    <t>Testpksyh</t>
+  </si>
+  <si>
+    <t>85142734</t>
+  </si>
+  <si>
+    <t>Autogardb</t>
+  </si>
+  <si>
+    <t>Testxlgmr</t>
+  </si>
+  <si>
+    <t>85142735</t>
+  </si>
+  <si>
+    <t>Autovyunz</t>
+  </si>
+  <si>
+    <t>Testrvtzb</t>
+  </si>
+  <si>
+    <t>85142736</t>
+  </si>
+  <si>
+    <t>Autoknqdm</t>
+  </si>
+  <si>
+    <t>Testezmia</t>
+  </si>
+  <si>
+    <t>85142737</t>
+  </si>
+  <si>
+    <t>Autobopcx</t>
+  </si>
+  <si>
+    <t>Testvtmsx</t>
+  </si>
+  <si>
+    <t>85142738</t>
+  </si>
+  <si>
+    <t>Autoeezrs</t>
+  </si>
+  <si>
+    <t>Testugfbf</t>
+  </si>
+  <si>
+    <t>32664756</t>
+  </si>
+  <si>
+    <t>85142814</t>
+  </si>
+  <si>
+    <t>85142816</t>
+  </si>
+  <si>
+    <t>85142817</t>
+  </si>
+  <si>
+    <t>Autobodgy</t>
+  </si>
+  <si>
+    <t>Testkmlxs</t>
+  </si>
+  <si>
+    <t>85142818</t>
   </si>
 </sst>
 </file>
@@ -1564,10 +1693,10 @@
         <v>223</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>258</v>
+        <v>303</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>243</v>
+        <v>300</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>15</v>
@@ -1600,10 +1729,10 @@
         <v>226</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>237</v>
+        <v>295</v>
       </c>
       <c r="O2" t="s" s="0">
-        <v>238</v>
+        <v>296</v>
       </c>
       <c r="P2" t="s" s="0">
         <v>227</v>
@@ -2013,16 +2142,16 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>15</v>

</xml_diff>

<commit_message>
B2B Form7 Tests Included
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/backup_testData.xlsx
+++ b/src/test/resources/data/BAT/backup_testData.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80A7960F-AB54-4A98-BF81-28F5BF5AFFC6}"/>
+  <xr:revisionPtr revIDLastSave="227" documentId="13_ncr:1_{A3C00A53-B60F-4FFA-AC45-FA356BAFF82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F2E7D06-F925-432E-825C-6568E02A2511}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GWCC" sheetId="1" r:id="rId1"/>
-    <sheet name="eForm7_PI" sheetId="7" r:id="rId2"/>
-    <sheet name="eForm6_PI" sheetId="2" r:id="rId3"/>
-    <sheet name="eForm6_Illness" sheetId="3" r:id="rId4"/>
-    <sheet name="eForm6_Mental" sheetId="4" r:id="rId5"/>
-    <sheet name="eForm6_Construction" sheetId="5" r:id="rId6"/>
-    <sheet name="eForm6_Other" sheetId="6" r:id="rId7"/>
+    <sheet name="B2BForm7" sheetId="8" r:id="rId2"/>
+    <sheet name="eForm7_PI" sheetId="7" r:id="rId3"/>
+    <sheet name="eForm6_PI" sheetId="2" r:id="rId4"/>
+    <sheet name="eForm6_Illness" sheetId="3" r:id="rId5"/>
+    <sheet name="eForm6_Mental" sheetId="4" r:id="rId6"/>
+    <sheet name="eForm6_Construction" sheetId="5" r:id="rId7"/>
+    <sheet name="eForm6_Other" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3206" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="247">
   <si>
     <t>ReferenceNumber</t>
   </si>
@@ -569,12 +570,6 @@
     <t>01/May/1992</t>
   </si>
   <si>
-    <t>32664493</t>
-  </si>
-  <si>
-    <t>938808</t>
-  </si>
-  <si>
     <t>Account Number</t>
   </si>
   <si>
@@ -749,228 +744,55 @@
     <t>1/Mar/2024</t>
   </si>
   <si>
-    <t>85142631</t>
-  </si>
-  <si>
-    <t>85142652</t>
-  </si>
-  <si>
-    <t>Autodcmqi</t>
-  </si>
-  <si>
-    <t>Testbtezw</t>
-  </si>
-  <si>
-    <t>85142653</t>
-  </si>
-  <si>
-    <t>85142655</t>
-  </si>
-  <si>
-    <t>Autowfsdb</t>
-  </si>
-  <si>
-    <t>Testhlwmg</t>
-  </si>
-  <si>
-    <t>32664620</t>
-  </si>
-  <si>
-    <t>85142660</t>
-  </si>
-  <si>
-    <t>32664631</t>
-  </si>
-  <si>
-    <t>575821</t>
-  </si>
-  <si>
-    <t>85142662</t>
-  </si>
-  <si>
-    <t>32664635</t>
-  </si>
-  <si>
-    <t>060368</t>
-  </si>
-  <si>
-    <t>85142664</t>
-  </si>
-  <si>
-    <t>32664638</t>
-  </si>
-  <si>
-    <t>237627</t>
-  </si>
-  <si>
-    <t>85142665</t>
-  </si>
-  <si>
-    <t>85142667</t>
-  </si>
-  <si>
-    <t>32664643</t>
-  </si>
-  <si>
-    <t>590865</t>
-  </si>
-  <si>
-    <t>85142668</t>
-  </si>
-  <si>
-    <t>85142669</t>
-  </si>
-  <si>
-    <t>Autolsvqq</t>
-  </si>
-  <si>
-    <t>Testveaou</t>
-  </si>
-  <si>
-    <t>85142670</t>
-  </si>
-  <si>
-    <t>32664651</t>
-  </si>
-  <si>
-    <t>301850</t>
-  </si>
-  <si>
-    <t>85142671</t>
-  </si>
-  <si>
-    <t>Autoybkzz</t>
-  </si>
-  <si>
-    <t>Testpnlry</t>
-  </si>
-  <si>
-    <t>85142697</t>
-  </si>
-  <si>
-    <t>85142698</t>
-  </si>
-  <si>
-    <t>85142699</t>
-  </si>
-  <si>
-    <t>85142700</t>
-  </si>
-  <si>
-    <t>Autosxtdx</t>
-  </si>
-  <si>
-    <t>Testjjtni</t>
-  </si>
-  <si>
-    <t>85142703</t>
-  </si>
-  <si>
     <t>32664708</t>
   </si>
   <si>
     <t>993630</t>
   </si>
   <si>
-    <t>85142716</t>
-  </si>
-  <si>
-    <t>Autoglyvm</t>
-  </si>
-  <si>
-    <t>Testkskic</t>
-  </si>
-  <si>
-    <t>85142727</t>
-  </si>
-  <si>
-    <t>Autopafdk</t>
-  </si>
-  <si>
-    <t>Testpmrkf</t>
-  </si>
-  <si>
-    <t>85142730</t>
-  </si>
-  <si>
-    <t>Autoxabxq</t>
-  </si>
-  <si>
-    <t>Testpksyh</t>
-  </si>
-  <si>
-    <t>85142734</t>
-  </si>
-  <si>
-    <t>Autogardb</t>
-  </si>
-  <si>
-    <t>Testxlgmr</t>
-  </si>
-  <si>
-    <t>85142735</t>
-  </si>
-  <si>
-    <t>Autovyunz</t>
-  </si>
-  <si>
-    <t>Testrvtzb</t>
-  </si>
-  <si>
-    <t>85142736</t>
-  </si>
-  <si>
-    <t>Autoknqdm</t>
-  </si>
-  <si>
-    <t>Testezmia</t>
-  </si>
-  <si>
-    <t>85142737</t>
-  </si>
-  <si>
     <t>Autobopcx</t>
   </si>
   <si>
     <t>Testvtmsx</t>
   </si>
   <si>
-    <t>85142738</t>
-  </si>
-  <si>
-    <t>Autoeezrs</t>
-  </si>
-  <si>
-    <t>Testugfbf</t>
-  </si>
-  <si>
     <t>32664756</t>
   </si>
   <si>
-    <t>85142814</t>
-  </si>
-  <si>
-    <t>85142816</t>
-  </si>
-  <si>
     <t>85142817</t>
   </si>
   <si>
-    <t>Autobodgy</t>
-  </si>
-  <si>
-    <t>Testkmlxs</t>
-  </si>
-  <si>
-    <t>85142818</t>
+    <t>85142819</t>
+  </si>
+  <si>
+    <t>accountNumber</t>
+  </si>
+  <si>
+    <t>Firstuydja</t>
+  </si>
+  <si>
+    <t>Lastxuxdu</t>
+  </si>
+  <si>
+    <t>3978262</t>
+  </si>
+  <si>
+    <t>Mon Jan 01 00:00:00 EST 1990</t>
+  </si>
+  <si>
+    <t>Firstjpmtk</t>
+  </si>
+  <si>
+    <t>Lastbxbuy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/mmm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="d/mmm/yyyy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -1009,12 +831,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1515,6 +1338,50 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68879496-E29C-4870-9412-2C416A5C3163}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="15.28515625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.28515625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.5703125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="10.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s" s="0">
+        <v>240</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C054F313-B8A2-4709-8028-7C8E0478B7C1}">
   <dimension ref="A1:AR2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1556,7 +1423,7 @@
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1565,138 +1432,138 @@
         <v>154</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F1" t="s" s="0">
         <v>16</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="I1" t="s" s="0">
         <v>84</v>
       </c>
       <c r="J1" t="s" s="0">
+        <v>182</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>183</v>
+      </c>
+      <c r="L1" t="s" s="0">
         <v>184</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="M1" t="s" s="0">
         <v>185</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="N1" t="s" s="0">
         <v>186</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="O1" t="s" s="0">
         <v>187</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="P1" t="s" s="0">
         <v>188</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="Q1" t="s" s="0">
         <v>189</v>
-      </c>
-      <c r="P1" t="s" s="0">
-        <v>190</v>
-      </c>
-      <c r="Q1" t="s" s="0">
-        <v>191</v>
       </c>
       <c r="R1" t="s" s="0">
         <v>9</v>
       </c>
       <c r="S1" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="T1" t="s" s="0">
+        <v>191</v>
+      </c>
+      <c r="U1" t="s" s="0">
         <v>192</v>
-      </c>
-      <c r="T1" t="s" s="0">
-        <v>193</v>
-      </c>
-      <c r="U1" t="s" s="0">
-        <v>194</v>
       </c>
       <c r="V1" t="s" s="0">
         <v>12</v>
       </c>
       <c r="W1" t="s" s="0">
+        <v>194</v>
+      </c>
+      <c r="X1" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="Y1" t="s" s="0">
         <v>196</v>
       </c>
-      <c r="X1" t="s" s="0">
+      <c r="Z1" t="s" s="0">
         <v>197</v>
       </c>
-      <c r="Y1" t="s" s="0">
-        <v>198</v>
-      </c>
-      <c r="Z1" t="s" s="0">
+      <c r="AA1" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="AB1" t="s" s="0">
         <v>199</v>
       </c>
-      <c r="AA1" t="s" s="0">
+      <c r="AC1" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="AD1" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="AE1" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="AF1" t="s" s="0">
         <v>205</v>
       </c>
-      <c r="AB1" t="s" s="0">
-        <v>201</v>
-      </c>
-      <c r="AC1" t="s" s="0">
-        <v>202</v>
-      </c>
-      <c r="AD1" t="s" s="0">
-        <v>203</v>
-      </c>
-      <c r="AE1" t="s" s="0">
-        <v>204</v>
-      </c>
-      <c r="AF1" t="s" s="0">
+      <c r="AG1" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="AH1" t="s" s="0">
         <v>207</v>
       </c>
-      <c r="AG1" t="s" s="0">
-        <v>208</v>
-      </c>
-      <c r="AH1" t="s" s="0">
+      <c r="AI1" t="s" s="0">
         <v>209</v>
       </c>
-      <c r="AI1" t="s" s="0">
-        <v>211</v>
-      </c>
       <c r="AJ1" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="AK1" t="s" s="0">
         <v>212</v>
       </c>
-      <c r="AK1" t="s" s="0">
+      <c r="AL1" t="s" s="0">
+        <v>213</v>
+      </c>
+      <c r="AM1" t="s" s="0">
         <v>214</v>
       </c>
-      <c r="AL1" t="s" s="0">
+      <c r="AN1" t="s" s="0">
         <v>215</v>
       </c>
-      <c r="AM1" t="s" s="0">
+      <c r="AO1" t="s" s="0">
         <v>216</v>
       </c>
-      <c r="AN1" t="s" s="0">
+      <c r="AP1" t="s" s="0">
         <v>217</v>
       </c>
-      <c r="AO1" t="s" s="0">
+      <c r="AQ1" t="s" s="0">
         <v>218</v>
       </c>
-      <c r="AP1" t="s" s="0">
-        <v>219</v>
-      </c>
-      <c r="AQ1" t="s" s="0">
+      <c r="AR1" t="s" s="0">
         <v>220</v>
-      </c>
-      <c r="AR1" t="s" s="0">
-        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>303</v>
+        <v>238</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>15</v>
@@ -1711,31 +1578,31 @@
         <v>18</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J2" t="s" s="0">
+        <v>222</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="N2" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="O2" t="s" s="0">
+        <v>236</v>
+      </c>
+      <c r="P2" t="s" s="0">
         <v>225</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="N2" t="s" s="0">
-        <v>295</v>
-      </c>
-      <c r="O2" t="s" s="0">
-        <v>296</v>
-      </c>
-      <c r="P2" t="s" s="0">
-        <v>227</v>
       </c>
       <c r="Q2" t="s" s="0">
         <v>23</v>
@@ -1744,7 +1611,7 @@
         <v>22</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="T2" t="s" s="0">
         <v>26</v>
@@ -1753,22 +1620,22 @@
         <v>157</v>
       </c>
       <c r="V2" t="s" s="0">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="W2" t="s" s="0">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="Z2" t="s" s="0">
         <v>24</v>
       </c>
       <c r="AA2" t="s" s="0">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="AB2" t="s" s="0">
         <v>138</v>
@@ -1786,16 +1653,16 @@
         <v>43</v>
       </c>
       <c r="AG2" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="AH2" t="s" s="0">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="AI2" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="AJ2" t="s" s="0">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="AK2" t="s" s="0">
         <v>138</v>
@@ -1810,13 +1677,13 @@
         <v>138</v>
       </c>
       <c r="AO2" t="s" s="0">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="AP2" t="s" s="0">
         <v>138</v>
       </c>
       <c r="AQ2" t="s" s="0">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="AR2" t="s" s="0">
         <v>138</v>
@@ -1830,7 +1697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33828E7C-EAC4-4C86-87E0-3EB8DC303443}">
   <dimension ref="A1:BY2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2142,16 +2009,16 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>306</v>
+        <v>239</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>274</v>
+        <v>233</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>158</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>275</v>
+        <v>234</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>15</v>
@@ -2391,7 +2258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64E6A5F-66F3-47EA-9AEB-61CD493B9923}">
   <dimension ref="A1:BW2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2937,7 +2804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D26FBA-7439-42B9-A201-C3C27FE83F69}">
   <dimension ref="A1:BX2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3492,7 +3359,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{047E5626-4C4D-4FFC-85FB-69A376807120}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3747,7 +3614,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673F62D1-C22D-4ED7-B45C-1711D3211AD6}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>